<commit_message>
add: tien tro thang 7
</commit_message>
<xml_diff>
--- a/$/Money.xlsx
+++ b/$/Money.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\tro\$\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9E309262-BEC0-4CBA-A084-698211731E7C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{895B151F-A9F5-45F1-903E-8560B680E1F5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -566,15 +566,15 @@
         <v>2542</v>
       </c>
       <c r="H7" s="4">
-        <v>3000</v>
+        <v>2561</v>
       </c>
       <c r="I7" s="4">
         <f>IF(H7-G7 &gt; 0, H7-G7, 0)</f>
-        <v>458</v>
+        <v>19</v>
       </c>
       <c r="J7" s="7">
         <f>I7*3000</f>
-        <v>1374000</v>
+        <v>57000</v>
       </c>
       <c r="K7" s="4">
         <v>1</v>
@@ -585,7 +585,7 @@
       </c>
       <c r="M7" s="8">
         <f>F7+J7+L7</f>
-        <v>3984000</v>
+        <v>2667000</v>
       </c>
       <c r="N7" s="4">
         <v>2500000</v>
@@ -601,14 +601,16 @@
       <c r="G8" s="4">
         <v>3736</v>
       </c>
-      <c r="H8" s="4"/>
+      <c r="H8" s="4">
+        <v>3946</v>
+      </c>
       <c r="I8" s="4">
         <f t="shared" ref="I8:I20" si="0">IF(H8-G8 &gt; 0, H8-G8, 0)</f>
-        <v>0</v>
+        <v>210</v>
       </c>
       <c r="J8" s="7">
         <f t="shared" ref="J8:J20" si="1">I8*3000</f>
-        <v>0</v>
+        <v>630000</v>
       </c>
       <c r="K8" s="4">
         <v>1</v>
@@ -619,7 +621,7 @@
       </c>
       <c r="M8" s="8">
         <f t="shared" ref="M8:M20" si="3">F8+J8+L8</f>
-        <v>3310000</v>
+        <v>3940000</v>
       </c>
       <c r="N8" s="4">
         <v>3000000</v>
@@ -630,19 +632,21 @@
         <v>201</v>
       </c>
       <c r="F9" s="7">
-        <v>3000000</v>
+        <v>3300000</v>
       </c>
       <c r="G9" s="4">
         <v>5894</v>
       </c>
-      <c r="H9" s="4"/>
+      <c r="H9" s="4">
+        <v>6085</v>
+      </c>
       <c r="I9" s="4">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>191</v>
       </c>
       <c r="J9" s="7">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>573000</v>
       </c>
       <c r="K9" s="4">
         <v>2</v>
@@ -653,7 +657,7 @@
       </c>
       <c r="M9" s="8">
         <f t="shared" si="3"/>
-        <v>3220000</v>
+        <v>4093000</v>
       </c>
       <c r="N9" s="4">
         <v>2800000</v>
@@ -669,14 +673,16 @@
       <c r="G10" s="4">
         <v>5826</v>
       </c>
-      <c r="H10" s="4"/>
+      <c r="H10" s="4">
+        <v>5951</v>
+      </c>
       <c r="I10" s="4">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>125</v>
       </c>
       <c r="J10" s="7">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>375000</v>
       </c>
       <c r="K10" s="4">
         <v>2</v>
@@ -687,7 +693,7 @@
       </c>
       <c r="M10" s="8">
         <f t="shared" si="3"/>
-        <v>3020000</v>
+        <v>3395000</v>
       </c>
       <c r="N10" s="4">
         <v>2800000</v>
@@ -703,14 +709,16 @@
       <c r="G11" s="4">
         <v>7113</v>
       </c>
-      <c r="H11" s="4"/>
+      <c r="H11" s="4">
+        <v>7240</v>
+      </c>
       <c r="I11" s="4">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>127</v>
       </c>
       <c r="J11" s="7">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>381000</v>
       </c>
       <c r="K11" s="4">
         <v>1</v>
@@ -721,7 +729,7 @@
       </c>
       <c r="M11" s="8">
         <f t="shared" si="3"/>
-        <v>3110000</v>
+        <v>3491000</v>
       </c>
       <c r="N11" s="4">
         <v>3000000</v>
@@ -737,14 +745,16 @@
       <c r="G12" s="4">
         <v>14308</v>
       </c>
-      <c r="H12" s="4"/>
+      <c r="H12" s="4">
+        <v>14848</v>
+      </c>
       <c r="I12" s="4">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>540</v>
       </c>
       <c r="J12" s="7">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>1620000</v>
       </c>
       <c r="K12" s="4">
         <v>2</v>
@@ -755,7 +765,7 @@
       </c>
       <c r="M12" s="8">
         <f t="shared" si="3"/>
-        <v>3420000</v>
+        <v>5040000</v>
       </c>
       <c r="N12" s="4">
         <v>2800000</v>
@@ -771,14 +781,16 @@
       <c r="G13" s="4">
         <v>6034</v>
       </c>
-      <c r="H13" s="4"/>
+      <c r="H13" s="4">
+        <v>6286</v>
+      </c>
       <c r="I13" s="4">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>252</v>
       </c>
       <c r="J13" s="7">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>756000</v>
       </c>
       <c r="K13" s="4">
         <v>1</v>
@@ -789,7 +801,7 @@
       </c>
       <c r="M13" s="8">
         <f t="shared" si="3"/>
-        <v>3210000</v>
+        <v>3966000</v>
       </c>
       <c r="N13" s="4">
         <v>3100000</v>
@@ -805,14 +817,16 @@
       <c r="G14" s="4">
         <v>6821</v>
       </c>
-      <c r="H14" s="4"/>
+      <c r="H14" s="4">
+        <v>6985</v>
+      </c>
       <c r="I14" s="4">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>164</v>
       </c>
       <c r="J14" s="7">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>492000</v>
       </c>
       <c r="K14" s="4">
         <v>1</v>
@@ -823,7 +837,7 @@
       </c>
       <c r="M14" s="8">
         <f t="shared" si="3"/>
-        <v>3010000</v>
+        <v>3502000</v>
       </c>
       <c r="N14" s="4">
         <v>2900000</v>
@@ -839,14 +853,16 @@
       <c r="G15" s="4">
         <v>7758</v>
       </c>
-      <c r="H15" s="4"/>
+      <c r="H15" s="4">
+        <v>7980</v>
+      </c>
       <c r="I15" s="4">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>222</v>
       </c>
       <c r="J15" s="7">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>666000</v>
       </c>
       <c r="K15" s="4">
         <v>2</v>
@@ -857,7 +873,7 @@
       </c>
       <c r="M15" s="8">
         <f t="shared" si="3"/>
-        <v>3220000</v>
+        <v>3886000</v>
       </c>
       <c r="N15" s="4">
         <v>3000000</v>
@@ -868,19 +884,21 @@
         <v>304</v>
       </c>
       <c r="F16" s="7">
-        <v>2900000</v>
+        <v>3200000</v>
       </c>
       <c r="G16" s="4">
         <v>6688</v>
       </c>
-      <c r="H16" s="4"/>
+      <c r="H16" s="4">
+        <v>6768</v>
+      </c>
       <c r="I16" s="4">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>80</v>
       </c>
       <c r="J16" s="7">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>240000</v>
       </c>
       <c r="K16" s="4">
         <v>1</v>
@@ -891,10 +909,10 @@
       </c>
       <c r="M16" s="8">
         <f t="shared" si="3"/>
-        <v>3010000</v>
+        <v>3550000</v>
       </c>
       <c r="N16" s="4">
-        <v>2500000</v>
+        <v>3200000</v>
       </c>
     </row>
     <row r="17" spans="5:14" x14ac:dyDescent="0.25">
@@ -907,14 +925,16 @@
       <c r="G17" s="4">
         <v>1763</v>
       </c>
-      <c r="H17" s="4"/>
+      <c r="H17" s="4">
+        <v>2182</v>
+      </c>
       <c r="I17" s="4">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>419</v>
       </c>
       <c r="J17" s="7">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>1257000</v>
       </c>
       <c r="K17" s="4">
         <v>2</v>
@@ -925,7 +945,7 @@
       </c>
       <c r="M17" s="8">
         <f t="shared" si="3"/>
-        <v>3220000</v>
+        <v>4477000</v>
       </c>
       <c r="N17" s="4">
         <v>2500000</v>
@@ -941,14 +961,16 @@
       <c r="G18" s="4">
         <v>5359</v>
       </c>
-      <c r="H18" s="4"/>
+      <c r="H18" s="4">
+        <v>5474</v>
+      </c>
       <c r="I18" s="4">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>115</v>
       </c>
       <c r="J18" s="7">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>345000</v>
       </c>
       <c r="K18" s="4">
         <v>1</v>
@@ -959,7 +981,7 @@
       </c>
       <c r="M18" s="8">
         <f t="shared" si="3"/>
-        <v>2910000</v>
+        <v>3255000</v>
       </c>
       <c r="N18" s="4">
         <v>2800000</v>
@@ -975,14 +997,16 @@
       <c r="G19" s="4">
         <v>609</v>
       </c>
-      <c r="H19" s="4"/>
+      <c r="H19" s="4">
+        <v>755</v>
+      </c>
       <c r="I19" s="4">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>146</v>
       </c>
       <c r="J19" s="7">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>438000</v>
       </c>
       <c r="K19" s="4">
         <v>2</v>
@@ -993,7 +1017,7 @@
       </c>
       <c r="M19" s="8">
         <f t="shared" si="3"/>
-        <v>3120000</v>
+        <v>3558000</v>
       </c>
       <c r="N19" s="4">
         <v>2300000</v>
@@ -1009,14 +1033,16 @@
       <c r="G20" s="4">
         <v>6993</v>
       </c>
-      <c r="H20" s="4"/>
+      <c r="H20" s="4">
+        <v>7160</v>
+      </c>
       <c r="I20" s="4">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>167</v>
       </c>
       <c r="J20" s="7">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>501000</v>
       </c>
       <c r="K20" s="4">
         <v>1</v>
@@ -1027,7 +1053,7 @@
       </c>
       <c r="M20" s="8">
         <f t="shared" si="3"/>
-        <v>3010000</v>
+        <v>3511000</v>
       </c>
       <c r="N20" s="4">
         <v>2300000</v>
@@ -1039,7 +1065,7 @@
       </c>
       <c r="F21" s="6">
         <f>SUM(F7:F20)</f>
-        <v>41200000</v>
+        <v>41800000</v>
       </c>
       <c r="G21" s="6">
         <f t="shared" ref="G21:N21" si="4">SUM(G7:G20)</f>
@@ -1047,15 +1073,15 @@
       </c>
       <c r="H21" s="6">
         <f t="shared" si="4"/>
-        <v>3000</v>
+        <v>84221</v>
       </c>
       <c r="I21" s="6">
         <f t="shared" si="4"/>
-        <v>458</v>
+        <v>2777</v>
       </c>
       <c r="J21" s="6">
         <f t="shared" si="4"/>
-        <v>1374000</v>
+        <v>8331000</v>
       </c>
       <c r="K21" s="6">
         <f t="shared" si="4"/>
@@ -1067,11 +1093,11 @@
       </c>
       <c r="M21" s="6">
         <f>F21+J21+L21</f>
-        <v>44774000</v>
+        <v>52331000</v>
       </c>
       <c r="N21" s="6">
         <f t="shared" si="4"/>
-        <v>38300000</v>
+        <v>39000000</v>
       </c>
     </row>
     <row r="22" spans="5:14" x14ac:dyDescent="0.25">
@@ -1080,7 +1106,7 @@
       </c>
       <c r="F22" s="6">
         <f>SUM(F7:F20)</f>
-        <v>41200000</v>
+        <v>41800000</v>
       </c>
       <c r="G22" s="6">
         <f t="shared" ref="G22:N22" si="5">SUM(G7:G20)</f>
@@ -1088,15 +1114,15 @@
       </c>
       <c r="H22" s="6">
         <f t="shared" si="5"/>
-        <v>3000</v>
+        <v>84221</v>
       </c>
       <c r="I22" s="6">
         <f t="shared" si="5"/>
-        <v>458</v>
+        <v>2777</v>
       </c>
       <c r="J22" s="6">
         <f t="shared" si="5"/>
-        <v>1374000</v>
+        <v>8331000</v>
       </c>
       <c r="K22" s="6">
         <f t="shared" si="5"/>
@@ -1108,11 +1134,11 @@
       </c>
       <c r="M22" s="6">
         <f t="shared" si="5"/>
-        <v>44774000</v>
+        <v>52331000</v>
       </c>
       <c r="N22" s="6">
         <f t="shared" si="5"/>
-        <v>38300000</v>
+        <v>39000000</v>
       </c>
     </row>
   </sheetData>
@@ -1124,12 +1150,12 @@
     <filterColumn colId="6" showButton="0"/>
   </autoFilter>
   <mergeCells count="6">
+    <mergeCell ref="N5:N6"/>
     <mergeCell ref="E4:M4"/>
     <mergeCell ref="E5:F5"/>
     <mergeCell ref="G5:J5"/>
     <mergeCell ref="K5:L5"/>
     <mergeCell ref="M5:M6"/>
-    <mergeCell ref="N5:N6"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>